<commit_message>
Fixed permission issue  (#205)
* fixed permission issue (#237)

* Update forms to 4.x (#238)

---------

Co-authored-by: iesmail-znz <49481318+iesmail-znz@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/forms/app/chv_youth_peer_education.xlsx
+++ b/forms/app/chv_youth_peer_education.xlsx
@@ -11,14 +11,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion1">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataSignature="AMtx7mjwEIOTpwB6N+NNriffcy6zo9+06g=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataSignature="AMtx7mhwNajzAWbnnBtKUQCWoeuCIfp0jA=="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="215">
   <si>
     <t>type</t>
   </si>
@@ -725,7 +725,6 @@
     <font>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -796,9 +795,6 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
     <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
@@ -810,6 +806,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
@@ -1520,7 +1519,7 @@
       <c r="B17" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="3" t="s">
         <v>23</v>
       </c>
       <c r="D17" s="3"/>
@@ -1911,7 +1910,7 @@
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
-      <c r="L29" s="9" t="s">
+      <c r="L29" s="8" t="s">
         <v>100</v>
       </c>
       <c r="M29" s="3"/>
@@ -2072,7 +2071,7 @@
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
-      <c r="L34" s="9" t="s">
+      <c r="L34" s="8" t="s">
         <v>118</v>
       </c>
       <c r="M34" s="3"/>
@@ -2122,31 +2121,31 @@
       <c r="C36" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="D36" s="9" t="s">
         <v>124</v>
       </c>
       <c r="E36" s="3"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="10"/>
-      <c r="K36" s="10"/>
-      <c r="L36" s="11"/>
-      <c r="M36" s="10"/>
-      <c r="N36" s="10"/>
-      <c r="O36" s="10"/>
-      <c r="P36" s="10"/>
-      <c r="Q36" s="10"/>
-      <c r="R36" s="10"/>
-      <c r="S36" s="10"/>
-      <c r="T36" s="10"/>
-      <c r="U36" s="10"/>
-      <c r="V36" s="10"/>
-      <c r="W36" s="10"/>
-      <c r="X36" s="10"/>
-      <c r="Y36" s="10"/>
-      <c r="Z36" s="10"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="10"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
+      <c r="Y36" s="9"/>
+      <c r="Z36" s="9"/>
     </row>
     <row r="37" ht="36.0" customHeight="1">
       <c r="A37" s="3" t="s">
@@ -2359,7 +2358,7 @@
       <c r="C45" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D45" s="12" t="s">
+      <c r="D45" s="11" t="s">
         <v>146</v>
       </c>
       <c r="E45" s="3"/>
@@ -2388,7 +2387,7 @@
       <c r="C46" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="D46" s="12" t="s">
+      <c r="D46" s="11" t="s">
         <v>150</v>
       </c>
       <c r="E46" s="3" t="s">
@@ -2417,7 +2416,7 @@
       <c r="C47" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="D47" s="12" t="s">
+      <c r="D47" s="11" t="s">
         <v>153</v>
       </c>
       <c r="E47" s="3" t="s">
@@ -2454,7 +2453,7 @@
       <c r="C48" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="D48" s="12" t="s">
+      <c r="D48" s="11" t="s">
         <v>160</v>
       </c>
       <c r="E48" s="3" t="s">
@@ -2489,7 +2488,7 @@
         <v>164</v>
       </c>
       <c r="C49" s="3"/>
-      <c r="D49" s="12"/>
+      <c r="D49" s="11"/>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -2515,7 +2514,7 @@
       <c r="C50" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D50" s="12" t="s">
+      <c r="D50" s="11" t="s">
         <v>168</v>
       </c>
       <c r="E50" s="3"/>
@@ -2570,7 +2569,7 @@
         <v>171</v>
       </c>
       <c r="C52" s="3"/>
-      <c r="D52" s="12" t="s">
+      <c r="D52" s="11" t="s">
         <v>172</v>
       </c>
       <c r="E52" s="3"/>
@@ -2597,7 +2596,7 @@
         <v>144</v>
       </c>
       <c r="C53" s="3"/>
-      <c r="D53" s="12"/>
+      <c r="D53" s="11"/>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -2622,12 +2621,14 @@
       <c r="C54" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D54" s="12" t="s">
+      <c r="D54" s="11" t="s">
         <v>176</v>
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
+      <c r="G54" s="12" t="s">
+        <v>48</v>
+      </c>
       <c r="H54" s="3"/>
       <c r="I54" s="3"/>
       <c r="J54" s="3"/>
@@ -2676,7 +2677,7 @@
       <c r="C56" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D56" s="12" t="s">
+      <c r="D56" s="11" t="s">
         <v>182</v>
       </c>
       <c r="E56" s="3" t="s">
@@ -2722,7 +2723,7 @@
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
-      <c r="D58" s="12"/>
+      <c r="D58" s="11"/>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
       <c r="G58" s="3"/>
@@ -2741,7 +2742,7 @@
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="13"/>
-      <c r="D59" s="12"/>
+      <c r="D59" s="11"/>
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
@@ -2775,13 +2776,13 @@
       <c r="P60" s="3"/>
       <c r="Q60" s="3"/>
       <c r="R60" s="3"/>
-      <c r="S60" s="11"/>
+      <c r="S60" s="10"/>
     </row>
     <row r="61" ht="36.0" customHeight="1">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
-      <c r="D61" s="12"/>
+      <c r="D61" s="11"/>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
@@ -2800,7 +2801,7 @@
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
-      <c r="D62" s="12"/>
+      <c r="D62" s="11"/>
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
       <c r="G62" s="3"/>
@@ -2819,7 +2820,7 @@
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
-      <c r="D63" s="12"/>
+      <c r="D63" s="11"/>
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
       <c r="G63" s="3"/>
@@ -2859,7 +2860,7 @@
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
-      <c r="D65" s="12"/>
+      <c r="D65" s="11"/>
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
       <c r="G65" s="3"/>
@@ -2878,7 +2879,7 @@
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
-      <c r="D66" s="12"/>
+      <c r="D66" s="11"/>
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
       <c r="G66" s="3"/>
@@ -2897,7 +2898,7 @@
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
-      <c r="D67" s="12"/>
+      <c r="D67" s="11"/>
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
@@ -2916,7 +2917,7 @@
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
-      <c r="D68" s="12"/>
+      <c r="D68" s="11"/>
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
       <c r="G68" s="3"/>
@@ -5868,7 +5869,7 @@
       </c>
       <c r="C2" s="15" t="str">
         <f>TEXT(NOW(), "yyyy-mm-dd_HH-MM")</f>
-        <v>2022-11-04_01-00</v>
+        <v>2023-03-07_03-39</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>213</v>

</xml_diff>